<commit_message>
Corrida | SFE-GNAC | 2026-04-07 08:22:24.602176
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GNAC_out.xlsx
+++ b/indicadores/SFE-GNAC_out.xlsx
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">06/04/2026</t>
+    <t xml:space="preserve">07/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">ysonder</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2173,7 +2173,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00147328201112221</v>
+        <v>0.00144263532955197</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2203,7 +2203,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.285163797525526</v>
+        <v>0.285107855227591</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -25064,13 +25064,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58BD2100-9676-455F-A6EC-52674C50BFE6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C40CC06-809A-4EC3-B19D-D539DE4BC317}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AFFECD8-3A5A-4D3B-95B3-46895E62B2FE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D8C7E42-880F-4E03-BFB2-A361BC8CB739}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB988396-FD0D-4C07-B8B5-21571CB10D75}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6432464-4C41-4365-BE69-088A3D9920AF}"/>
 </file>
</xml_diff>